<commit_message>
Show each test case's summary on its own sheet
The test case template has a new Summary row under Test Case ID, and
fill_template.py fills it from the case's title - the same words as the
Summary sheet's Title column - so a tester reading one sheet knows what
it checks.

Applies to workbooks built from now on. Existing workbooks are left as
they are: rebuilding one would add the row but wipe recorded execution
results. SKILL.md says how to write the summary.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/.claude/skills/generate-test-cases/Test_Case_Template.xlsx
+++ b/.claude/skills/generate-test-cases/Test_Case_Template.xlsx
@@ -1,94 +1,45 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\krist\Documents\GitHub\IS212\.claude\skills\generate-test-cases\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0C833B1-3214-4950-B267-D1CA56A46BE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="TC01" sheetId="1" r:id="rId1"/>
+    <sheet name="TC01" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="13">
-  <si>
-    <t>Item</t>
-  </si>
-  <si>
-    <t>Test Case ID</t>
-  </si>
-  <si>
-    <t>Pre-conditions</t>
-  </si>
-  <si>
-    <t>Test Steps</t>
-  </si>
-  <si>
-    <t>Test Data</t>
-  </si>
-  <si>
-    <t>Expected Result</t>
-  </si>
-  <si>
-    <t>Created By</t>
-  </si>
-  <si>
-    <t>Creation Date</t>
-  </si>
-  <si>
-    <t>Actual Result</t>
-  </si>
-  <si>
-    <t>Pass/Fail/Not Executed/Blocked</t>
-  </si>
-  <si>
-    <t>Remarks</t>
-  </si>
-  <si>
-    <t>Executed by</t>
-  </si>
-  <si>
-    <t>Date of Execution</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="3">
     <font>
+      <name val="Arial"/>
+      <color rgb="FF000000"/>
       <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color theme="1"/>
       <sz val="10"/>
-      <color theme="1"/>
-      <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Arial"/>
+      <color theme="1"/>
       <sz val="10"/>
-      <color theme="1"/>
-      <name val="Arial"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -134,27 +85,86 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="7">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -355,101 +365,139 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
-  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C16"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="24.77734375" customWidth="1"/>
-    <col min="2" max="2" width="56.77734375" customWidth="1"/>
+    <col width="24.77734375" customWidth="1" min="1" max="1"/>
+    <col width="56.77734375" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2"/>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="3"/>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3" s="3"/>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" s="3"/>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B5" s="3"/>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B6" s="3"/>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B7" s="3"/>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B8" s="3"/>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="B10" s="5"/>
-      <c r="C10" s="6"/>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B11" s="3"/>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B12" s="3"/>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B13" s="3"/>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="B14" s="3"/>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B15" s="3"/>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Pre-conditions</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Test Steps</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Creation Date</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n"/>
+    </row>
+    <row r="10"/>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n"/>
+      <c r="C11" s="6" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Date of Execution</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Docs: generator writes the Status columns and Commit row; README says how to start a workbook
fill_template.py adds Status (default Active), Superseded by and Change # to
the Summary sheet from optional per-case JSON fields, validates them, and
widens the title and Code reviewed bands to column I. The template's TC01
gets a Commit row in its execution block. SKILL.md documents the fields and
says to build a workbook from JSON only when it is new. docs/test-cases/
README.md points new stories at /generate-test-cases - the one source of the
layout - in place of a separate blank workbook (PR #72).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/.claude/skills/generate-test-cases/Test_Case_Template.xlsx
+++ b/.claude/skills/generate-test-cases/Test_Case_Template.xlsx
@@ -370,7 +370,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="24.77734375" customWidth="1" min="1" max="1"/>
@@ -449,7 +449,6 @@
       </c>
       <c r="B9" s="3" t="n"/>
     </row>
-    <row r="10"/>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -498,6 +497,14 @@
         </is>
       </c>
       <c r="B16" s="3" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>